<commit_message>
docs: record session 23; status workbook rebuilt; counts to 486
PROGRESS.md: the next actions are now all the owner's (public repos,
video, Railway/Vercel with SIGNER_TOKEN/KEEPER_PRIVATE_KEY/CORS_ORIGINS,
explorer key); B6 and B7 cleared; the demo commands pin BOTH brain chains
and unset the contracts .env's GEMINI_API_KEY, with the reason; decisions
appended, superseding the Sep 23 "on-chain cap" claim rather than
rewriting it; and a disclosure that two early runs this session sent
orchestrator requests to Gemini, none of which succeeded.

The status workbook is rebuilt from real per-file test counts (486), with
the Sep 29 defects, cleared blockers and what is outstanding. The deck and
the submission carry the same count.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,12 +55,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00A32020"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -108,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -143,9 +137,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -679,7 +670,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>15</v>
@@ -743,7 +734,7 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>7</v>
@@ -875,12 +866,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pnpm demo, M3 done-condition, 3 chaos items, backup video</t>
+          <t>pnpm demo, M3 done-condition, chaos items, backup video</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>No model key in agentx-backend/.env</t>
+          <t>No model</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -893,14 +884,14 @@
           <t>Sep 23</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Free GEMINI_API_KEY or GROQ_API_KEY. The agent loop has never run end to end with a real model; the last four defects all lived on that path.</t>
+          <t>Cleared Sep 29 with local Ollama (llama3 8B), no API quota. The first live runs found sixteen defects on the hire-to-settle path.</t>
         </is>
       </c>
     </row>
@@ -922,7 +913,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -930,14 +921,14 @@
           <t>Sep 23</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Routes return 200 and the API contract holds, but nothing has checked how it renders.</t>
+          <t>Rendered Sep 29 with headless Chrome. First render found the API sent no CORS headers, so every page said API unreachable; fixed.</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1242,15 +1233,15 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>agent-core/orchestrator</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Registration, discovery, hiring, job lifecycle, the error contract</t>
+          <t>Every failure branch, and the retry of a silent worker with another agent</t>
         </is>
       </c>
     </row>
@@ -1262,15 +1253,15 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>db/constraints</t>
+          <t>api</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Every documented database guarantee, tried by writing the bad row</t>
+          <t>Registration, discovery, hiring, idempotent retries, the earned fast path, auth codes</t>
         </is>
       </c>
     </row>
@@ -1282,15 +1273,15 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>agent-core/fallback</t>
+          <t>sdk/client</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Provider chain, automatic fall-through</t>
+          <t>Retries, idempotency keys, typed errors, NotAccepted</t>
         </is>
       </c>
     </row>
@@ -1302,15 +1293,15 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>agent-core/orchestrator</t>
+          <t>agent-core/worker</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Every failure branch: no candidate, budget, timeout, schema</t>
+          <t>Offer loop, decline, triage outage, retrying a transient accept</t>
         </is>
       </c>
     </row>
@@ -1326,11 +1317,11 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Untrusted-content containment</t>
+          <t>Untrusted-content containment; the judge's rating scale</t>
         </is>
       </c>
     </row>
@@ -1342,15 +1333,15 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>mcp/tools</t>
+          <t>api/chaos</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Tool descriptions, spend warnings, error retryability</t>
+          <t>Malformed result, daily cap, result shape, on-chain hash</t>
         </is>
       </c>
     </row>
@@ -1362,15 +1353,15 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>api/meta</t>
+          <t>signer</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Network and budget endpoints, secret-leak guard</t>
+          <t>Caps (on-chain and, for EOAs, off-chain), gas floor, replay, failed-broadcast recovery</t>
         </is>
       </c>
     </row>
@@ -1382,15 +1373,15 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>signer</t>
+          <t>db/constraints</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Caps, gas floor, replay, failed-broadcast recovery on the same nonce</t>
+          <t>Every documented database guarantee, tried by writing the bad row</t>
         </is>
       </c>
     </row>
@@ -1402,15 +1393,15 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>agent-core/worker</t>
+          <t>agent-core/fallback</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Offer loop, structural decline, self-check</t>
+          <t>Provider chain, cached replay, recorders sharing one file</t>
         </is>
       </c>
     </row>
@@ -1422,15 +1413,15 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>api/chaos</t>
+          <t>indexer/replay</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Malformed result, daily cap, result shape, on-chain hash</t>
+          <t>Replay safety, refund reasons, tx hashes, confidence floor, party-checked linking</t>
         </is>
       </c>
     </row>
@@ -1442,15 +1433,15 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>api/runs</t>
+          <t>api/meta</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Run lifecycle, durable trace, terminal state</t>
+          <t>Network and budget endpoints, the 24h rollover</t>
         </is>
       </c>
     </row>
@@ -1462,15 +1453,15 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>indexer/loop</t>
+          <t>mcp/tools</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Exponential backoff, recovery, clean shutdown</t>
+          <t>Tool descriptions, spend warnings, error retryability</t>
         </is>
       </c>
     </row>
@@ -1482,15 +1473,15 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>config/money</t>
+          <t>api/runs</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Base-unit formatting and parsing</t>
+          <t>Run lifecycle, durable trace, terminal state</t>
         </is>
       </c>
     </row>
@@ -1502,15 +1493,15 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>indexer/replay</t>
+          <t>indexer/loop</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Replay safety: a restart cannot manufacture reputation</t>
+          <t>Exponential backoff, recovery, clean shutdown</t>
         </is>
       </c>
     </row>
@@ -1522,46 +1513,186 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>mcp/server</t>
+          <t>signer/keeper</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>A real MCP session: schemas, annotations, tool errors</t>
+          <t>Which permissionless exit is due, at every deadline boundary</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>config/money</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Base-unit formatting and parsing</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>sdk/stream</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>SSE frames split at every byte offset; a bad frame does not end the stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>api/identity</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>ERC-8004 id verified against the registry before it is stored</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>mcp/server</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>A real MCP session: schemas, annotations, tool errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>signer/auth</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>SIGNER_TOKEN, loopback-only without one</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>api/cors</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>A browser on another origin can call the API; credentials stay off</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>api/submit</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>The API presents the signer token</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t>agentx-interface</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>lib/api</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C31" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>formatUnits, including exactness past 2^53</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="15" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C25" s="11">
-        <f>SUM(C2:C24)</f>
+      <c r="C32" s="11">
+        <f>SUM(C2:C31)</f>
         <v/>
       </c>
     </row>
@@ -1576,7 +1707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1956,6 +2087,402 @@
       <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>No demo job had ever settled: eight defects between hire and settlement, each hiding the next</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>First live runs, Sep 29</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Spending caps were enforced nowhere for EOA agents (all of them); the signer read AgentAccount, failed, and allowed</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>No process ever sent the escrow's permissionless exits; stranded money stayed stranded</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Fixed: keeper</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>A retried hire inserted a phantom job each time, backed by no transaction</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Live e2e, Sep 29</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>The indexer linked jobs by spec hash alone, crediting a worker for an old run's payment</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Live e2e, Sep 29</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Every refund, including a client's cancel, counted as the worker failing</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Agents registered through the API or /register could never be hired: nothing set chain_agent_id</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>The API sent no CORS headers; every browser request was refused</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>First browser render, Sep 29</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>fastPathMinScore was read by nothing; unproven workers were paid up front</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>The signer accepted signing requests from anyone who could reach it</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Fixed: token</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>The judge's 0-100 score came back on three scales; approved work was disputed</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Live runs, Sep 29</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Recorders sharing a cache file erased each other; a replay lost two of three steps</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Cached replay, Sep 29</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>A worker abandoned a job the API had told it to retry</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Mid-job chaos run, Sep 29</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>pnpm demo passed with one step of three settled</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Cached replay, Sep 29</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>/v1/budget ignored the 24h rollover</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Deploy ignored ARBITER_ADDRESS and FEE_RECIPIENT; make drift called a script that did not exist</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Indexer rewinds on a reorg but does not delete rows from orphaned blocks</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Documented</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>A disputed job has no timeout; only the arbiter can resolve it</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Documented</t>
         </is>
       </c>
     </row>
@@ -2010,71 +2537,71 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>pnpm demo has never run end to end</t>
+          <t>Hosted model key (optional now)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>User</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Blocked on a model key. This is M3's done-condition.</t>
+          <t>Local Ollama works; a Gemini or Groq key would improve judgement quality in the video. One is already in agentx-contracts/.env and was not used without asking.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Model provider key in agentx-backend/.env</t>
+          <t>Phone hotspot run</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Free tier: GEMINI_API_KEY or GROQ_API_KEY.</t>
+          <t>The one chaos item left: no baked-in timeout assumptions on a slow network.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Kill a worker mid-job; run on a phone hotspot</t>
+          <t>Railway (api, signer, indexer) + Vercel</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>User</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2084,19 +2611,19 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>The two chaos items that need a live run.</t>
+          <t>Set SIGNER_TOKEN in both API and signer, KEEPER_PRIVATE_KEY in the signer, CORS_ORIGINS in the API.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Submit</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Railway (api, signer, indexer) + Vercel</t>
+          <t>2-3 minute video</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -2111,24 +2638,24 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Deferred to M5 by the owner.</t>
+          <t>Record the cached replay (157 s) and the interface. Claude cannot record video.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Contracts</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Audit docs 01-04, 07, 10 against the code</t>
+          <t>Verify source on the explorer</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>User</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2138,7 +2665,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>This activity has found more defects than writing new code.</t>
+          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
         </is>
       </c>
     </row>
@@ -2150,22 +2677,22 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2-3 minute video</t>
+          <t>Make the three repos public</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>User</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Needs the demo to run first.</t>
+          <t>Required by Oct 13.</t>
         </is>
       </c>
     </row>
@@ -2177,12 +2704,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Verify source on the explorer</t>
+          <t>Move demo agents onto AgentAccount</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2192,34 +2719,34 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
+          <t>Turns the on-chain cap claim from design into fact; today the signer enforces caps for EOAs.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Interface</t>
+          <t>Indexer</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Open it in a browser and look at it</t>
+          <t>Delete rows from orphaned blocks on a reorg</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Either</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Never done. Routes 200, contract holds, rendering unverified.</t>
+          <t>Documented limitation; the indexer trails the head by the confirmation depth.</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2893,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record session 24; counts to 498; workbook rebuilt
PROGRESS.md records the orchestrator's AgentAccount and the
compromised-signer result, 7/7 chaos, the reorg handling and the run
history, with new decisions appended. Nothing left that is Claude's to
do before the deadline; what remains is the owner's (public repos,
video, hosting, explorer key) or post-hackathon.

Test counts recounted by the JSON reporter — 128 + 363 + 7 = 498 — in
the deck, the submission, the overview and the status workbook, whose
Tests sheet sums to the same number.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>7</v>
@@ -1357,11 +1357,11 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Caps (on-chain and, for EOAs, off-chain), gas floor, replay, failed-broadcast recovery</t>
+          <t>AgentAccount routing via execute, caps on- and off-chain, gas, replay, stranded-nonce release, error classification</t>
         </is>
       </c>
     </row>
@@ -1417,11 +1417,11 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Replay safety, refund reasons, tx hashes, confidence floor, party-checked linking</t>
+          <t>Replay safety, refund reasons, tx hashes, confidence floor, party-checked linking, reorgs</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2445,42 +2445,108 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Indexer rewinds on a reorg but does not delete rows from orphaned blocks</t>
+          <t>After a reorg a re-mined settlement was credited twice and a dropped one kept forever</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Docs audit, Sep 29</t>
+          <t>Reorg review, Sep 29</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Documented</t>
+          <t>Fixed: dedupe + halt</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>No agent used AgentAccount, so the on-chain cap claim held for nothing</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Docs audit, Sep 29</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Fixed: orchestrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>A failed broadcast's nonce claim blocked every later request as in flight</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>AgentAccount live run</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>An empty gas wallet was reported as an unreachable RPC (503 matched inside tx hex)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>AgentAccount live run</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>A disputed job has no timeout; only the arbiter can resolve it</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Docs audit, Sep 29</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Documented</t>
         </is>
@@ -2497,7 +2563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2564,39 +2630,39 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Phone hotspot run</t>
+          <t>Railway (api, signer, indexer) + Vercel</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>User</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>The one chaos item left: no baked-in timeout assumptions on a slow network.</t>
+          <t>Set SIGNER_TOKEN in both API and signer, KEEPER_PRIVATE_KEY in the signer, CORS_ORIGINS in the API.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Submit</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Railway (api, signer, indexer) + Vercel</t>
+          <t>2-3 minute video</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2611,19 +2677,19 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Set SIGNER_TOKEN in both API and signer, KEEPER_PRIVATE_KEY in the signer, CORS_ORIGINS in the API.</t>
+          <t>Record the cached replay (157 s) and the interface. Claude cannot record video.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Submit</t>
+          <t>Contracts</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2-3 minute video</t>
+          <t>Verify source on the explorer</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -2638,19 +2704,19 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Record the cached replay (157 s) and the interface. Claude cannot record video.</t>
+          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Contracts</t>
+          <t>Submit</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Verify source on the explorer</t>
+          <t>Make the three repos public</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2660,51 +2726,51 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
+          <t>Required by Oct 13.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Submit</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Make the three repos public</t>
+          <t>Give workers AgentAccounts too</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Required by Oct 13.</t>
+          <t>Workers never spend today; only needed if one ever pays another agent.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Contracts</t>
+          <t>Stretch</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Move demo agents onto AgentAccount</t>
+          <t>x402 facilitator</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2714,24 +2780,24 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Turns the on-chain cap claim from design into fact; today the signer enforces caps for EOAs.</t>
+          <t>First to be cut.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Indexer</t>
+          <t>Post-hack</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Delete rows from orphaned blocks on a reorg</t>
+          <t>Map TaskEscrow onto the ERC-8183 Job interface</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -2741,91 +2807,10 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Documented limitation; the indexer trails the head by the confirmation depth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Interface</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Runs history page</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>/v1/runs exists; nothing renders it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>x402 facilitator</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>First to be cut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Post-hack</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Map TaskEscrow onto the ERC-8183 Job interface</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Explicitly out of scope before the deadline.</t>
         </is>

</xml_diff>

<commit_message>
docs: record session 25; counts to 536; workbook and deck rebuilt
PROGRESS: header and next actions (everything left is yours: repos public,
the video, testnet MON for it, hosting, explorer key); the stale Sep 25
status section rewritten; M3 15/15; four decisions; the session entry; new
gotchas — local ephemeral-port exhaustion (the old meta.test.ts "flake"),
Git Bash globs through $TEMP, and a demo run's ~0.5 MON cost.

Keeper, live: chain job 149, stranded by the mid-job chaos run, went
ACCEPTED → expireUndelivered → REFUNDED at its deadline.

Workbook: 536 tests from real per-file counts, eight defects found today, the
outstanding list. Deck: 536, 150 s, every demo agent on an AgentAccount, and
"workers are plain wallets" replaced by the honest x402 limitation — slides
5 and 10 rendered through PowerPoint and inspected.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -664,13 +664,13 @@
           <t>Oct 3-5</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>15</v>
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1237,11 +1237,11 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Every failure branch, and the retry of a silent worker with another agent</t>
+          <t>Every failure branch, the retry of a silent worker, never hiring itself, a model outage mid-selection</t>
         </is>
       </c>
     </row>
@@ -1253,15 +1253,15 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>api/x402</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Registration, discovery, hiring, idempotent retries, the earned fast path, auth codes</t>
+          <t>Facilitator: settle, verify, redeem once, every forged or mismatched receipt refused against the chain</t>
         </is>
       </c>
     </row>
@@ -1273,15 +1273,15 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>sdk/client</t>
+          <t>api</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Retries, idempotency keys, typed errors, NotAccepted</t>
+          <t>Registration, discovery, hiring, idempotent retries, the earned fast path, auth codes</t>
         </is>
       </c>
     </row>
@@ -1293,15 +1293,15 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>agent-core/worker</t>
+          <t>sdk/client</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Offer loop, decline, triage outage, retrying a transient accept</t>
+          <t>Retries, idempotency keys, typed errors, NotAccepted</t>
         </is>
       </c>
     </row>
@@ -1313,15 +1313,15 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>agent-core/injection</t>
+          <t>agent-core/worker</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Untrusted-content containment; the judge's rating scale</t>
+          <t>Offer loop, decline, triage outage, retrying a transient accept</t>
         </is>
       </c>
     </row>
@@ -1333,15 +1333,15 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>api/chaos</t>
+          <t>agent-core/x402</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Malformed result, daily cap, result shape, on-chain hash</t>
+          <t>Paid endpoint: 402 quote, redeem before work, waits for confirmation, job loop skips x402 jobs</t>
         </is>
       </c>
     </row>
@@ -1353,15 +1353,15 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>signer</t>
+          <t>agent-core/injection</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>AgentAccount routing via execute, caps on- and off-chain, gas, replay, stranded-nonce release, error classification</t>
+          <t>Untrusted-content containment; the judge's rating scale</t>
         </is>
       </c>
     </row>
@@ -1373,15 +1373,15 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>db/constraints</t>
+          <t>api/chaos</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Every documented database guarantee, tried by writing the bad row</t>
+          <t>Malformed result, daily cap, result shape, on-chain hash</t>
         </is>
       </c>
     </row>
@@ -1393,15 +1393,15 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>agent-core/fallback</t>
+          <t>signer</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Provider chain, cached replay, recorders sharing one file</t>
+          <t>AgentAccount routing via execute (the key the account granted), caps on- and off-chain, gas, replay, stranded-nonce release, error classification</t>
         </is>
       </c>
     </row>
@@ -1413,15 +1413,15 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>indexer/replay</t>
+          <t>db/constraints</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Replay safety, refund reasons, tx hashes, confidence floor, party-checked linking, reorgs</t>
+          <t>Every documented database guarantee, tried by writing the bad row</t>
         </is>
       </c>
     </row>
@@ -1433,15 +1433,15 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>api/meta</t>
+          <t>agent-core/fallback</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Network and budget endpoints, the 24h rollover</t>
+          <t>Provider chain, cached replay, recorders sharing one file, provider detail kept, no key in a URL</t>
         </is>
       </c>
     </row>
@@ -1453,15 +1453,15 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>mcp/tools</t>
+          <t>indexer/replay</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Tool descriptions, spend warnings, error retryability</t>
+          <t>Replay safety, refund reasons, tx hashes, confidence floor, party-checked linking, reorgs</t>
         </is>
       </c>
     </row>
@@ -1473,15 +1473,15 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>api/runs</t>
+          <t>api/meta</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Run lifecycle, durable trace, terminal state</t>
+          <t>Network and budget endpoints, the 24h rollover</t>
         </is>
       </c>
     </row>
@@ -1493,15 +1493,15 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>indexer/loop</t>
+          <t>mcp/tools</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Exponential backoff, recovery, clean shutdown</t>
+          <t>Tool descriptions, spend warnings, error retryability</t>
         </is>
       </c>
     </row>
@@ -1513,15 +1513,15 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>signer/keeper</t>
+          <t>api/runs</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Which permissionless exit is due, at every deadline boundary</t>
+          <t>Run lifecycle, durable trace, terminal state</t>
         </is>
       </c>
     </row>
@@ -1533,15 +1533,15 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>config/money</t>
+          <t>indexer/loop</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Base-unit formatting and parsing</t>
+          <t>Exponential backoff, recovery, clean shutdown</t>
         </is>
       </c>
     </row>
@@ -1553,15 +1553,15 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>sdk/stream</t>
+          <t>signer/keeper</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>SSE frames split at every byte offset; a bad frame does not end the stream</t>
+          <t>Which permissionless exit is due, at every deadline boundary</t>
         </is>
       </c>
     </row>
@@ -1573,15 +1573,15 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>api/identity</t>
+          <t>config/money</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>ERC-8004 id verified against the registry before it is stored</t>
+          <t>Base-unit formatting and parsing</t>
         </is>
       </c>
     </row>
@@ -1593,15 +1593,15 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>mcp/server</t>
+          <t>sdk/stream</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>A real MCP session: schemas, annotations, tool errors</t>
+          <t>SSE frames split at every byte offset; a bad frame does not end the stream</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>signer/auth</t>
+          <t>api/identity</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>SIGNER_TOKEN, loopback-only without one</t>
+          <t>ERC-8004 id verified against the registry before it is stored</t>
         </is>
       </c>
     </row>
@@ -1633,15 +1633,15 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>api/cors</t>
+          <t>mcp/server</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>A browser on another origin can call the API; credentials stay off</t>
+          <t>A real MCP session: schemas, annotations, tool errors</t>
         </is>
       </c>
     </row>
@@ -1653,46 +1653,86 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>api/submit</t>
+          <t>signer/auth</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>The API presents the signer token</t>
+          <t>SIGNER_TOKEN, loopback-only without one</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>api/cors</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>A browser on another origin can call the API; credentials stay off</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>api/submit</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>The API presents the signer token</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t>agentx-interface</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>lib/api</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C33" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>formatUnits, including exactness past 2^53</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="14" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C32" s="11">
-        <f>SUM(C2:C31)</f>
+      <c r="C34" s="11">
+        <f>SUM(C2:C33)</f>
         <v/>
       </c>
     </row>
@@ -1707,7 +1747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2549,6 +2589,182 @@
       <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Documented</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>The orchestrator offered its own capability to the planner and tried to hire itself</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Mid-job chaos run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>A model outage while choosing an agent aborted the whole run instead of ending the step</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Why a plan failed was discarded; every cause read as 'could not reach a model'</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>The default Gemini model was retired (404); Session 23's Gemini failures were likely this</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Fixed: gemini-3.8-flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>The Gemini key travelled in the URL query string</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Fixed: header</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>The demo reused a CREATE2 salt after an aborted run; createAccount reverted</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>The demo harness did not survive a dropped broadcast; one injected 503 aborted it</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Slow-RPC chaos, Sep 30</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Fixed: resend signed bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>The live run page would never have shown a plan-failed event (no SSE listener)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Review, Sep 30</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2603,12 +2819,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Hosted model key (optional now)</t>
+          <t>Railway (api, signer, indexer) + Vercel</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2618,24 +2834,24 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Local Ollama works; a Gemini or Groq key would improve judgement quality in the video. One is already in agentx-contracts/.env and was not used without asking.</t>
+          <t>Set SIGNER_TOKEN in both API and signer, KEEPER_PRIVATE_KEY in the signer, CORS_ORIGINS in the API.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Submit</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Railway (api, signer, indexer) + Vercel</t>
+          <t>2-3 minute video</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -2650,19 +2866,19 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Set SIGNER_TOKEN in both API and signer, KEEPER_PRIVATE_KEY in the signer, CORS_ORIGINS in the API.</t>
+          <t>Record the cached replay (150 s, Ollama recording of Sep 30, with x402 and worker accounts) and the interface. Claude cannot record video.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Submit</t>
+          <t>Contracts</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2-3 minute video</t>
+          <t>Verify source on the explorer</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2677,19 +2893,19 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Record the cached replay (157 s) and the interface. Claude cannot record video.</t>
+          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Contracts</t>
+          <t>Submit</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Verify source on the explorer</t>
+          <t>Make the three repos public</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -2699,24 +2915,24 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
+          <t>Required by Oct 13. Full-history scan for every real secret: clean (Sep 30).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Submit</t>
+          <t>Testnet</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Make the three repos public</t>
+          <t>Testnet MON for the video run</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2726,24 +2942,24 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Required by Oct 13.</t>
+          <t>A demo run now costs ~0.5 MON. DEPLOYER ~0.36, FUNDER ~3.05 after Sep 30; AGENT_A/B hold 10 each, untouched.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Post-hack</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Give workers AgentAccounts too</t>
+          <t>ERC-8183 conformance: new kernel + AGENTX evaluator + hook; DISPUTED timeout</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -2753,66 +2969,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Workers never spend today; only needed if one ever pays another agent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Stretch</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>x402 facilitator</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>First to be cut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Post-hack</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Map TaskEscrow onto the ERC-8183 Job interface</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Explicitly out of scope before the deadline.</t>
+          <t>Mapping written: docs/12. Needs a redeploy, so after the deadline.</t>
         </is>
       </c>
     </row>
@@ -2878,7 +3040,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Session 26 wrap-up and Session 27 — v2 live checks, chaos at 20%
PROGRESS, overview, submission, deck and status workbook brought to v2:
addresses, 695 tests (184 · 471 · 40), the Session 26 hardening, the
20%-lossy chaos runs and the two defects they found, verify-indexer on
v2, and wallet balances (DEPLOYER nearly empty — top up before the video).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1093,15 +1093,15 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>TaskEscrow</t>
+          <t>AgentAccount</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Job state machine, settlement, fee split, the three permissionless exits</t>
+          <t>Caps, per-(target, selector) allowlist, forbidden approve-style selectors, session keys, two-step ownership, sweepNative</t>
         </is>
       </c>
     </row>
@@ -1113,15 +1113,15 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>AgentAccount</t>
+          <t>TaskEscrow</t>
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Spending caps, allowlists, session key lifetime, access control</t>
+          <t>Job state machine, settlement, fee split, the permissionless exits</t>
         </is>
       </c>
     </row>
@@ -1133,15 +1133,15 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>StakeVault</t>
+          <t>Guards</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Bonds per agent id, withdrawal delay, slashing</t>
+          <t>Reverts and boundary conditions</t>
         </is>
       </c>
     </row>
@@ -1153,15 +1153,15 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Adversarial</t>
+          <t>V2Findings</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Hostile sequences against the escrow</t>
+          <t>The Sep 30 audit findings, each failing on v1: SameOwner, dust, trapped payouts, dispute expiry, bounds, admin delay</t>
         </is>
       </c>
     </row>
@@ -1173,15 +1173,15 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Guards</t>
+          <t>V2Guards</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Reverts and boundary conditions</t>
+          <t>Every new guard branch in v2</t>
         </is>
       </c>
     </row>
@@ -1193,15 +1193,15 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Escrow.invariant</t>
+          <t>Adversarial</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Solvency, lockedTotal, fee bounds, no self-dealing (512k transitions each)</t>
+          <t>Hostile sequences against the escrow</t>
         </is>
       </c>
     </row>
@@ -1213,95 +1213,95 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MockUSDC</t>
+          <t>StakeVault</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Test token</t>
+          <t>Bonds per agent id, withdrawal delay, slashing to a recipient</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>agentx-backend</t>
+          <t>agentx-contracts</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>agent-core/orchestrator</t>
+          <t>Escrow.invariant</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Every failure branch, the retry of a silent worker, never hiring itself, a model outage mid-selection</t>
+          <t>Solvency = locked + owed, fees, disputes, pause, mid-flight params</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>agentx-backend</t>
+          <t>agentx-contracts</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>api/x402</t>
+          <t>StakeVault.invariant</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Facilitator: settle, verify, redeem once, every forged or mismatched receipt refused against the chain</t>
+          <t>Vault balance always covers bonds</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>agentx-backend</t>
+          <t>agentx-contracts</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>AgentAccount.invariant</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Registration, discovery, hiring, idempotent retries, the earned fast path, auth codes</t>
+          <t>No spend past a cap, no escape from the allowlist</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>agentx-backend</t>
+          <t>agentx-contracts</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>sdk/client</t>
+          <t>MockUSDC</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Retries, idempotency keys, typed errors, NotAccepted</t>
+          <t>Test token</t>
         </is>
       </c>
     </row>
@@ -1313,15 +1313,15 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>agent-core/worker</t>
+          <t>signer</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Offer loop, decline, triage outage, retrying a transient accept</t>
+          <t>AgentAccount routing, caps, gas, replay, nonce release, the advisory lock released on one connection, named contract refusals, an HTTP 503 is retryable</t>
         </is>
       </c>
     </row>
@@ -1333,15 +1333,15 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>agent-core/x402</t>
+          <t>agent-core/orchestrator</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Paid endpoint: 402 quote, redeem before work, waits for confirmation, job loop skips x402 jobs</t>
+          <t>Every failure branch, retrying a silent worker, a late accept waited for, never hiring itself, a model outage mid-selection</t>
         </is>
       </c>
     </row>
@@ -1353,15 +1353,15 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>agent-core/injection</t>
+          <t>api</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Untrusted-content containment; the judge's rating scale</t>
+          <t>Registration, discovery, hiring, idempotent retries, the earned fast path, uuid public ids</t>
         </is>
       </c>
     </row>
@@ -1373,15 +1373,15 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>api/chaos</t>
+          <t>agent-core/worker</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Malformed result, daily cap, result shape, on-chain hash</t>
+          <t>Offer loop, decline, transient accept, a failed submit retried without re-accepting</t>
         </is>
       </c>
     </row>
@@ -1393,15 +1393,15 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>signer</t>
+          <t>sdk/client</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>AgentAccount routing via execute (the key the account granted), caps on- and off-chain, gas, replay, stranded-nonce release, error classification</t>
+          <t>Retries, idempotency keys, typed errors, NotAccepted</t>
         </is>
       </c>
     </row>
@@ -1413,15 +1413,15 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>db/constraints</t>
+          <t>agent-core/fallback</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Every documented database guarantee, tried by writing the bad row</t>
+          <t>Provider chain, cached replay and its pacing cap, recorders, no key in a URL</t>
         </is>
       </c>
     </row>
@@ -1433,15 +1433,15 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>agent-core/fallback</t>
+          <t>api/x402</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Provider chain, cached replay, recorders sharing one file, provider detail kept, no key in a URL</t>
+          <t>Facilitator: settle, verify, redeem once, every forged receipt refused against the chain</t>
         </is>
       </c>
     </row>
@@ -1457,11 +1457,11 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Replay safety, refund reasons, tx hashes, confidence floor, party-checked linking, reorgs</t>
+          <t>Replay safety, v2 events, unresolved disputes earn nothing, reorgs, RPC blips are not reorgs</t>
         </is>
       </c>
     </row>
@@ -1473,15 +1473,15 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>api/meta</t>
+          <t>agent-core/injection</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Network and budget endpoints, the 24h rollover</t>
+          <t>Untrusted-content containment; the judge's rating scale</t>
         </is>
       </c>
     </row>
@@ -1493,15 +1493,15 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>mcp/tools</t>
+          <t>api/chaos</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Tool descriptions, spend warnings, error retryability</t>
+          <t>Malformed result, daily cap, result shape, on-chain hash</t>
         </is>
       </c>
     </row>
@@ -1513,15 +1513,15 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>api/runs</t>
+          <t>db/constraints</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Run lifecycle, durable trace, terminal state</t>
+          <t>Every documented database guarantee, tried by writing the bad row</t>
         </is>
       </c>
     </row>
@@ -1533,15 +1533,15 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>indexer/loop</t>
+          <t>api/meta</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Exponential backoff, recovery, clean shutdown</t>
+          <t>Network and budget endpoints, v2 parameters, the 24h rollover</t>
         </is>
       </c>
     </row>
@@ -1553,15 +1553,15 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>signer/keeper</t>
+          <t>mcp/tools</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Which permissionless exit is due, at every deadline boundary</t>
+          <t>Tool descriptions, spend warnings, error retryability</t>
         </is>
       </c>
     </row>
@@ -1573,15 +1573,15 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>config/money</t>
+          <t>api/endpoints</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Base-unit formatting and parsing</t>
+          <t>Readiness, metrics, public-https endpoints, 404 on serial ids</t>
         </is>
       </c>
     </row>
@@ -1593,15 +1593,15 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>sdk/stream</t>
+          <t>api/runs</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>SSE frames split at every byte offset; a bad frame does not end the stream</t>
+          <t>Run lifecycle, durable trace, terminal state</t>
         </is>
       </c>
     </row>
@@ -1613,15 +1613,15 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>api/identity</t>
+          <t>signer/app</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>ERC-8004 id verified against the registry before it is stored</t>
+          <t>Validated /sign, RFC 7807, no internal message in a 500</t>
         </is>
       </c>
     </row>
@@ -1633,15 +1633,15 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>mcp/server</t>
+          <t>signer/keeper</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>A real MCP session: schemas, annotations, tool errors</t>
+          <t>Which exit is due at every deadline, including expireDispute</t>
         </is>
       </c>
     </row>
@@ -1653,15 +1653,15 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>signer/auth</t>
+          <t>service</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>SIGNER_TOKEN, loopback-only without one</t>
+          <t>Env validation, bearer compare, timeouts, shutdown, metrics</t>
         </is>
       </c>
     </row>
@@ -1673,15 +1673,15 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>api/cors</t>
+          <t>indexer/loop</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>A browser on another origin can call the API; credentials stay off</t>
+          <t>Backoff, recovery, clean shutdown</t>
         </is>
       </c>
     </row>
@@ -1693,46 +1693,286 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>api/submit</t>
+          <t>config/money</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>The API presents the signer token</t>
+          <t>Base-unit formatting and parsing</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>sdk/stream</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>SSE frames split at every byte offset</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>agent-core/x402</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Paid endpoint: 402 quote, redeem before work</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>api/hardening</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Helmet, body limit, SSE cap, rate limit before auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>api/identity</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>ERC-8004 id verified against the registry before it is stored</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>api/submit</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Signer token, timeout, an unreachable signer is a retryable outage</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>mcp/server</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>A real MCP session: schemas, annotations, tool errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>signer/auth</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>SIGNER_TOKEN, loopback-only without one</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>api/cors</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Cross-origin browser calls; credentials stay off</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>agentx-backend</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>api/auth</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>ax_&lt;keyId&gt;_&lt;secret&gt;, one indexed lookup, legacy keys</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>agentx-interface</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>lib/api</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>formatUnits, including exactness past 2^53</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>lib/api + subscribe</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>formatUnits past 2^53; SSE kinds, bad frames, terminal close</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>lib/links</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Explorer links: https + known host only; uuid and agent id parsing</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>components</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>RunTrace (hostile links, money, live region), NetworkBadge (never assumes testnet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>lib/wallet</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Addresses and RPC validated before the wallet is asked; chain added on 4902</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C34" s="11">
-        <f>SUM(C2:C33)</f>
+      <c r="C46" s="11">
+        <f>SUM(C2:C45)</f>
         <v/>
       </c>
     </row>
@@ -1747,7 +1987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2578,7 +2818,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>A disputed job has no timeout; only the arbiter can resolve it</t>
+          <t>A disputed job had no timeout; only the arbiter could resolve it</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2588,24 +2828,24 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Documented</t>
+          <t>Fixed in v2: expireDispute</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>The orchestrator offered its own capability to the planner and tried to hire itself</t>
+          <t>The signer's per-agent advisory lock could stay held forever (taken and released on different pooled connections)</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Mid-job chaos run, Sep 30</t>
+          <t>Session 26 audit; reproduced in a test</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -2617,152 +2857,416 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>A model outage while choosing an agent aborted the whole run instead of ending the step</t>
+          <t>API auth ran scrypt against every stored key on every request: 12.9 s per request at a few hundred keys</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Gemini live run, Sep 30</t>
+          <t>Session 26 audit</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Fixed: keyId + SHA-256</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Why a plan failed was discarded; every cause read as 'could not reach a model'</t>
+          <t>Reputation farming by self-hire; a payout to a bad wallet trapped the job</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Gemini live run, Sep 30</t>
+          <t>Contract audit, Sep 30</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Fixed in v2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>The default Gemini model was retired (404); Session 23's Gemini failures were likely this</t>
+          <t>Jobs and runs were enumerable by serial id</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Gemini live run, Sep 30</t>
+          <t>Session 26 audit</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Fixed: gemini-3.8-flash</t>
+          <t>Fixed: uuid public ids</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>The Gemini key travelled in the URL query string</t>
+          <t>A worker abandoned finished work when a submit failed transiently</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Gemini live run, Sep 30</t>
+          <t>Slow-RPC chaos run on v2</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Fixed: header</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>The demo reused a CREATE2 salt after an aborted run; createAccount reverted</t>
+          <t>Explorer links from the API went straight into href (a javascript: URL would run)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Live run, Sep 30</t>
+          <t>Interface audit, Sep 30</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Fixed: allowlist</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>The demo harness did not survive a dropped broadcast; one injected 503 aborted it</t>
+          <t>An HTTP 503 from the RPC was reported INVALID_STATE, so workers gave up accepts and finished submits</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Slow-RPC chaos, Sep 30</t>
+          <t>20%-lossy chaos run, Session 27</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Fixed: resend signed bytes</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>A late accept made the cancel fail and the orchestrator abandoned the delivery</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>20%-lossy chaos run, Session 27</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>An unreachable signer was reported as INSUFFICIENT_FUNDS</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Session 26 audit</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>The indexer halted on one RPC 503 as if for a reorg</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Session 26 audit</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>SSE sent no headers until the first 25 s heartbeat</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Test written for the audit</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>The demo registered workers' records under the wrong owner once they owned their identities</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>First live v2 run</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>The orchestrator offered its own capability to the planner and tried to hire itself</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Mid-job chaos run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>A model outage while choosing an agent aborted the whole run instead of ending the step</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Why a plan failed was discarded; every cause read as 'could not reach a model'</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>The default Gemini model was retired (404); Session 23's Gemini failures were likely this</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Fixed: gemini-3.8-flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>The Gemini key travelled in the URL query string</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Gemini live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Fixed: header</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>The demo reused a CREATE2 salt after an aborted run; createAccount reverted</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>The demo harness did not survive a dropped broadcast; one injected 503 aborted it</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Slow-RPC chaos, Sep 30</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Fixed: resend signed bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>The live run page would never have shown a plan-failed event (no SSE listener)</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Review, Sep 30</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2866,7 +3370,7 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Record the cached replay (150 s, Ollama recording of Sep 30, with x402 and worker accounts) and the interface. Claude cannot record video.</t>
+          <t>Record the cached replay (v2 Ollama recording of Sep 30; 162 s with AGENT_REPLAY_MAX_MS=2000) and the interface. Claude cannot record video.</t>
         </is>
       </c>
     </row>
@@ -2947,7 +3451,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>A demo run now costs ~0.5 MON. DEPLOYER ~0.36, FUNDER ~3.05 after Sep 30; AGENT_A/B hold 10 each, untouched.</t>
+          <t>A demo run costs ~0.5 MON. See PROGRESS for current balances; 6 MON each moved from AGENT_A/B for v2, as allowed.</t>
         </is>
       </c>
     </row>
@@ -2959,7 +3463,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>ERC-8183 conformance: new kernel + AGENTX evaluator + hook; DISPUTED timeout</t>
+          <t>ERC-8183 conformance: new kernel + AGENTX evaluator + hook</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3083,12 +3587,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TaskEscrow</t>
+          <t>TaskEscrow (v2)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>0x1b0959dfd32323e5a4749d5444c2e6435349027c</t>
+          <t>0x4feED0338761817417Fd1dDdFC8331D16AEB370D</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Session 27 — M5-06 met, deploy-ready from one repo, 699 tests
PROGRESS, PLAN (M5-06 done; M2-22/23 point at the runbook and the
deployment check), CHANGELOG, overview, submission, deck and workbook:
the indexer defect found by the timed runs, the Railway build that could
not have built, the three clean timed runs (149 / 153 / 168 s), the
deploy rehearsal, refreshed screenshots, and current balances.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -1457,11 +1457,11 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Replay safety, v2 events, unresolved disputes earn nothing, reorgs, RPC blips are not reorgs</t>
+          <t>Replay safety, v2 events, unresolved disputes earn nothing, reorgs, RPC blips are not reorgs, state only moves forward</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2972,17 +2972,17 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>An HTTP 503 from the RPC was reported INVALID_STATE, so workers gave up accepts and finished submits</t>
+          <t>The indexer walked a job state backwards; a delivered job read accepted and approve was refused</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>20%-lossy chaos run, Session 27</t>
+          <t>M5-06 timed runs, Session 27</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Fixed: forward-only projection</t>
         </is>
       </c>
     </row>
@@ -2994,34 +2994,34 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>A late accept made the cancel fail and the orchestrator abandoned the delivery</t>
+          <t>A Railway build could not have built: chain facts came from a sibling checkout</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>20%-lossy chaos run, Session 27</t>
+          <t>Deploy rehearsal, Session 27</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Fixed: chain/ + drift check</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>An unreachable signer was reported as INSUFFICIENT_FUNDS</t>
+          <t>An HTTP 503 from the RPC was reported INVALID_STATE, so workers gave up accepts and finished submits</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Session 26 audit</t>
+          <t>20%-lossy chaos run, Session 27</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -3033,17 +3033,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>The indexer halted on one RPC 503 as if for a reorg</t>
+          <t>A late accept made the cancel fail and the orchestrator abandoned the delivery</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Session 26 audit</t>
+          <t>20%-lossy chaos run, Session 27</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -3060,12 +3060,12 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>SSE sent no headers until the first 25 s heartbeat</t>
+          <t>An unreachable signer was reported as INSUFFICIENT_FUNDS</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Test written for the audit</t>
+          <t>Session 26 audit</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -3082,12 +3082,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>The demo registered workers' records under the wrong owner once they owned their identities</t>
+          <t>The indexer halted on one RPC 503 as if for a reorg</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>First live v2 run</t>
+          <t>Session 26 audit</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -3099,17 +3099,17 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>The orchestrator offered its own capability to the planner and tried to hire itself</t>
+          <t>SSE sent no headers until the first 25 s heartbeat</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Mid-job chaos run, Sep 30</t>
+          <t>Test written for the audit</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -3121,17 +3121,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>A model outage while choosing an agent aborted the whole run instead of ending the step</t>
+          <t>The demo registered workers' records under the wrong owner once they owned their identities</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Gemini live run, Sep 30</t>
+          <t>First live v2 run</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -3143,17 +3143,17 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Why a plan failed was discarded; every cause read as 'could not reach a model'</t>
+          <t>The orchestrator offered its own capability to the planner and tried to hire itself</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Gemini live run, Sep 30</t>
+          <t>Mid-job chaos run, Sep 30</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
@@ -3165,12 +3165,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>The default Gemini model was retired (404); Session 23's Gemini failures were likely this</t>
+          <t>A model outage while choosing an agent aborted the whole run instead of ending the step</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Fixed: gemini-3.8-flash</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>The Gemini key travelled in the URL query string</t>
+          <t>Why a plan failed was discarded; every cause read as 'could not reach a model'</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Fixed: header</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3214,17 +3214,17 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>The demo reused a CREATE2 salt after an aborted run; createAccount reverted</t>
+          <t>The default Gemini model was retired (404); Session 23's Gemini failures were likely this</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Live run, Sep 30</t>
+          <t>Gemini live run, Sep 30</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Fixed: gemini-3.8-flash</t>
         </is>
       </c>
     </row>
@@ -3236,37 +3236,81 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>The demo harness did not survive a dropped broadcast; one injected 503 aborted it</t>
+          <t>The Gemini key travelled in the URL query string</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Slow-RPC chaos, Sep 30</t>
+          <t>Gemini live run, Sep 30</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>Fixed: resend signed bytes</t>
+          <t>Fixed: header</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>The demo reused a CREATE2 salt after an aborted run; createAccount reverted</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Live run, Sep 30</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>The demo harness did not survive a dropped broadcast; one injected 503 aborted it</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Slow-RPC chaos, Sep 30</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Fixed: resend signed bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>The live run page would never have shown a plan-failed event (no SSE listener)</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Review, Sep 30</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -3343,7 +3387,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Set SIGNER_TOKEN in both API and signer, KEEPER_PRIVATE_KEY in the signer, CORS_ORIGINS in the API.</t>
+          <t>Follow docs/13-deploy.md; then node scripts/check-deployment.mjs &lt;api&gt; &lt;site&gt;.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Session 27 — modern UI, the 404 fix, 725 tests
PROGRESS (UI session entry, the audit review, owner operations decisions
in Next actions, counts), overview, submission, deck and workbook: 184
contracts + 496 backend + 45 interface = 725, plus 12 smoke tests. The
workbook's per-file rows now include the audit's new status and indexer
progress tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1657,11 +1657,11 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Env validation, bearer compare, timeouts, shutdown, metrics</t>
+          <t>Env validation, bearer compare, timeouts, shutdown, metrics, build metadata, token-gated /metrics</t>
         </is>
       </c>
     </row>
@@ -1673,15 +1673,15 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>indexer/loop</t>
+          <t>api/status</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Backoff, recovery, clean shutdown</t>
+          <t>Public /v1/status: states and numbers only, cached, bounded checks, indexer lag</t>
         </is>
       </c>
     </row>
@@ -1693,15 +1693,15 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>config/money</t>
+          <t>indexer/progress</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Base-unit formatting and parsing</t>
+          <t>Head, indexed-block and lag gauges</t>
         </is>
       </c>
     </row>
@@ -1713,15 +1713,15 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>sdk/stream</t>
+          <t>indexer/loop</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>SSE frames split at every byte offset</t>
+          <t>Backoff, recovery, clean shutdown</t>
         </is>
       </c>
     </row>
@@ -1733,15 +1733,15 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>agent-core/x402</t>
+          <t>config/money</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Paid endpoint: 402 quote, redeem before work</t>
+          <t>Base-unit formatting and parsing</t>
         </is>
       </c>
     </row>
@@ -1753,15 +1753,15 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>api/hardening</t>
+          <t>sdk/stream</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Helmet, body limit, SSE cap, rate limit before auth</t>
+          <t>SSE frames split at every byte offset</t>
         </is>
       </c>
     </row>
@@ -1773,15 +1773,15 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>api/identity</t>
+          <t>agent-core/x402</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>ERC-8004 id verified against the registry before it is stored</t>
+          <t>Paid endpoint: 402 quote, redeem before work</t>
         </is>
       </c>
     </row>
@@ -1793,15 +1793,15 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>api/submit</t>
+          <t>api/hardening</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Signer token, timeout, an unreachable signer is a retryable outage</t>
+          <t>Helmet, body limit, SSE cap, rate limit before auth; a non-numeric or unknown agent id is 404</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>mcp/server</t>
+          <t>api/identity</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>A real MCP session: schemas, annotations, tool errors</t>
+          <t>ERC-8004 id verified against the registry before it is stored</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>signer/auth</t>
+          <t>api/submit</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>SIGNER_TOKEN, loopback-only without one</t>
+          <t>Signer token, timeout, an unreachable signer is a retryable outage</t>
         </is>
       </c>
     </row>
@@ -1853,15 +1853,15 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>api/cors</t>
+          <t>mcp/server</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Cross-origin browser calls; credentials stay off</t>
+          <t>A real MCP session: schemas, annotations, tool errors</t>
         </is>
       </c>
     </row>
@@ -1873,55 +1873,55 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>api/auth</t>
+          <t>signer/auth</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>ax_&lt;keyId&gt;_&lt;secret&gt;, one indexed lookup, legacy keys</t>
+          <t>SIGNER_TOKEN, loopback-only without one</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>agentx-interface</t>
+          <t>agentx-backend</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>lib/api + subscribe</t>
+          <t>api/cors</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>formatUnits past 2^53; SSE kinds, bad frames, terminal close</t>
+          <t>Cross-origin browser calls; credentials stay off</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>agentx-interface</t>
+          <t>agentx-backend</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>lib/links</t>
+          <t>api/auth</t>
         </is>
       </c>
       <c r="C43" s="6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Explorer links: https + known host only; uuid and agent id parsing</t>
+          <t>ax_&lt;keyId&gt;_&lt;secret&gt;, one indexed lookup, legacy keys</t>
         </is>
       </c>
     </row>
@@ -1933,15 +1933,15 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>components</t>
+          <t>lib/api + subscribe</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>RunTrace (hostile links, money, live region), NetworkBadge (never assumes testnet)</t>
+          <t>formatUnits past 2^53; SSE kinds, bad frames, terminal close</t>
         </is>
       </c>
     </row>
@@ -1953,26 +1953,86 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
+          <t>lib/links</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Explorer links: https + known host only; uuid and agent id parsing</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>components</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>RunTrace (hostile links, money, live region), NetworkBadge (never assumes testnet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
           <t>lib/wallet</t>
         </is>
       </c>
-      <c r="C45" s="6" t="n">
+      <c r="C47" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>Addresses and RPC validated before the wallet is asked; chain added on 4902</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="14" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>lib/format</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Relative time and durations, refusing nonsense input</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C46" s="11">
-        <f>SUM(C2:C45)</f>
+      <c r="C49" s="11">
+        <f>SUM(C2:C48)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: demo identities carry ERC-8004 agent cards; PLAN in sync; Session 28
- scripts/lib/chain.mjs agentCardUri(): the demo registers its orchestrator
  and workers with a registration-v1 card as a data: URI instead of
  `ipfs://<label>` placeholders that resolved to nothing. Verified on
  Monad testnet: identity #146's Registered event decodes to the card.
- PLAN.md re-checked against the code: 54 rows ticked with evidence, 4 cut
  with the reason in the row (fallback registries, off-chain scoreOf, and
  M2-03's seeded history — fabricated reputation, see Decisions). 106/116
  in scope; every open task but the final docs pass is the owner's.
- README says it is live and where; PROGRESS (Session 28, decisions,
  730 tests), submission doc, deck and workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -131,12 +131,12 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -606,10 +606,10 @@
         </is>
       </c>
       <c r="E3" s="6" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G3" s="5">
         <f>IF(F3=0,0,E3/F3)</f>
@@ -632,16 +632,16 @@
           <t>Sep 29 - Oct 2</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Deploy left (you)</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5">
         <f>IF(F4=0,0,E4/F4)</f>
@@ -696,13 +696,13 @@
           <t>Oct 6-8</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Deploy left (you)</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>11</v>
@@ -728,9 +728,9 @@
           <t>Oct 9-11</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Video left (you)</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>8</v>
@@ -777,23 +777,23 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="11">
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="10">
         <f>SUM(E2:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="10">
         <f>SUM(F2:F8)</f>
         <v/>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="12">
         <f>IF(F9=0,0,E9/F9)</f>
         <v/>
       </c>
@@ -995,7 +995,7 @@
           <t>Sep 28</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2013,26 +2013,46 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
+          <t>lib/agent-card</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>ERC-8004 registration-v1 card and its data: URI, non-ASCII safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
           <t>lib/format</t>
         </is>
       </c>
-      <c r="C48" s="2" t="n">
+      <c r="C49" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>Relative time and durations, refusing nonsense input</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="14" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C49" s="11">
-        <f>SUM(C2:C48)</f>
+      <c r="C50" s="10">
+        <f>SUM(C2:C49)</f>
         <v/>
       </c>
     </row>
@@ -3648,7 +3668,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Session 30: counts, Railway blocker, hosted-run design in PROGRESS
- 766 tests (77 interface) + 62 browser tests, also run in Firefox, WebKit
  and two phones; README, overview, submission, workbook and deck updated.
- PROGRESS: Railway trial expired (deploy waits on a plan); what hosted
  live runs need — fresh random keys, a daily session-key renewal (24 h
  contract cap), hosted workers, a per-orchestrator run cap; the Session 30
  log; CHANGELOG entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -1957,11 +1957,11 @@
         </is>
       </c>
       <c r="C45" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>formatUnits past 2^53; SSE kinds, bad frames, terminal close; 5xx/503 read as sentences</t>
+          <t>formatUnits past 2^53; SSE kinds, bad frames; only a terminal event ends a run; reconnect + replay reset; 5xx/503 read as sentences</t>
         </is>
       </c>
     </row>

</xml_diff>